<commit_message>
Final course material, 24 Sept 2026
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MhLFYHdNRLpSBsLtxiJZNA
</commit_message>
<xml_diff>
--- a/2. Database Systems & Learning Analytics (2026)/Assignment/Review_Log_Template/LA_review_templates.xlsx
+++ b/2. Database Systems & Learning Analytics (2026)/Assignment/Review_Log_Template/LA_review_templates.xlsx
@@ -180,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -202,11 +202,55 @@
         <color rgb="00D3DDEB"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3DDEB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3DDEB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3DDEB"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00D3DDEB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3DDEB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00D3DDEB"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D3DDEB"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D3DDEB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -290,6 +334,8 @@
     <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -669,6 +715,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -677,7 +724,7 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Προαιρετικό εργαλείο για τη δική σας ανασκόπηση· δεν χρειάζεται ποτέ στο μάθημα. Ένα φύλλο για κάθε βήμα της ανασκόπησης. Ό,τι καταγράφετε εδώ μεταφέρεται στη Μεθοδολογία και στα Αποτελέσματα της εργασίας.</t>
+          <t>Προαιρετικό εργαλείο για τη δική σας ανασκόπηση. Ένα φύλλο για κάθε βήμα της ανασκόπησης. Ό,τι καταγράφετε εδώ μεταφέρεται στη Μεθοδολογία και στα Αποτελέσματα της εργασίας.</t>
         </is>
       </c>
     </row>
@@ -1007,6 +1054,7 @@
         <v/>
       </c>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
         <is>
@@ -1023,6 +1071,7 @@
       </c>
       <c r="B17" s="14" t="n"/>
     </row>
+    <row r="18"/>
     <row r="19" ht="62" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
@@ -1033,10 +1082,10 @@
         <f>IF(F232="","","TITLE-ABS-KEY("&amp;F232&amp;")"&amp;IF(B16="",""," AND PUBYEAR &gt; "&amp;(B16-1))&amp;IF(B17="",""," AND LANGUAGE("&amp;B17&amp;")"))</f>
         <v/>
       </c>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="16" t="n"/>
+      <c r="C19" s="41" t="n"/>
+      <c r="D19" s="41" t="n"/>
+      <c r="E19" s="41" t="n"/>
+      <c r="F19" s="42" t="n"/>
     </row>
     <row r="20" ht="62" customHeight="1">
       <c r="A20" s="12" t="inlineStr">
@@ -1048,10 +1097,10 @@
         <f>IF(F232="","",F232&amp;IF(B16="",""," pubyearmin:"&amp;B16))</f>
         <v/>
       </c>
-      <c r="C20" s="16" t="n"/>
-      <c r="D20" s="16" t="n"/>
-      <c r="E20" s="16" t="n"/>
-      <c r="F20" s="16" t="n"/>
+      <c r="C20" s="41" t="n"/>
+      <c r="D20" s="41" t="n"/>
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="42" t="n"/>
     </row>
     <row r="21" ht="62" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
@@ -1063,10 +1112,10 @@
         <f>IF(F232="","",F232)</f>
         <v/>
       </c>
-      <c r="C21" s="16" t="n"/>
-      <c r="D21" s="16" t="n"/>
-      <c r="E21" s="16" t="n"/>
-      <c r="F21" s="16" t="n"/>
+      <c r="C21" s="41" t="n"/>
+      <c r="D21" s="41" t="n"/>
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="42" t="n"/>
     </row>
     <row r="22" ht="44" customHeight="1">
       <c r="A22" s="17" t="inlineStr">
@@ -1078,11 +1127,12 @@
         <f>IF(F232="","","Αστερίσκοι: "&amp;SUMPRODUCT(LEN(B6:F13)-LEN(SUBSTITUTE(B6:F13,"*","")))&amp;" (το IEEE Xplore δέχεται έως 10 ανά αναζήτηση). "&amp;IF(SUMPRODUCT(--ISNUMBER(FIND("*",B6:F13)),--((ISNUMBER(FIND(" ",TRIM(B6:F13)))+ISNUMBER(FIND("-",B6:F13)))&gt;0))&gt;0,"ΠΡΟΣΟΧΗ: "&amp;SUMPRODUCT(--ISNUMBER(FIND("*",B6:F13)),--((ISNUMBER(FIND(" ",TRIM(B6:F13)))+ISNUMBER(FIND("-",B6:F13)))&gt;0))&amp;" όρος ή όροι έχουν αστερίσκο μέσα σε φράση ή μετά από ενωτικό. Στο ERIC δεν επιστρέφουν αποτελέσματα: γράψτε τις παραλλαγές ολόκληρες.","Κανένας αστερίσκος μέσα σε φράση ή μετά από ενωτικό."))</f>
         <v/>
       </c>
-      <c r="C22" s="16" t="n"/>
-      <c r="D22" s="16" t="n"/>
-      <c r="E22" s="16" t="n"/>
-      <c r="F22" s="16" t="n"/>
-    </row>
+      <c r="C22" s="41" t="n"/>
+      <c r="D22" s="41" t="n"/>
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="42" t="n"/>
+    </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="19" t="inlineStr">
         <is>
@@ -1305,6 +1355,7 @@
         <v/>
       </c>
     </row>
+    <row r="36"/>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
         <is>
@@ -1327,6 +1378,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="62" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
@@ -1337,10 +1389,10 @@
         <f>IF(F295="","","TITLE-ABS-KEY("&amp;F295&amp;")"&amp;IF(B37="",""," AND PUBYEAR &gt; "&amp;(B37-1))&amp;IF(B38="",""," AND LANGUAGE("&amp;B38&amp;")"))</f>
         <v/>
       </c>
-      <c r="C40" s="16" t="n"/>
-      <c r="D40" s="16" t="n"/>
-      <c r="E40" s="16" t="n"/>
-      <c r="F40" s="16" t="n"/>
+      <c r="C40" s="41" t="n"/>
+      <c r="D40" s="41" t="n"/>
+      <c r="E40" s="41" t="n"/>
+      <c r="F40" s="42" t="n"/>
     </row>
     <row r="41" ht="62" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
@@ -1352,10 +1404,10 @@
         <f>IF(F295="","",F295&amp;IF(B37="",""," pubyearmin:"&amp;B37))</f>
         <v/>
       </c>
-      <c r="C41" s="16" t="n"/>
-      <c r="D41" s="16" t="n"/>
-      <c r="E41" s="16" t="n"/>
-      <c r="F41" s="16" t="n"/>
+      <c r="C41" s="41" t="n"/>
+      <c r="D41" s="41" t="n"/>
+      <c r="E41" s="41" t="n"/>
+      <c r="F41" s="42" t="n"/>
     </row>
     <row r="42" ht="62" customHeight="1">
       <c r="A42" s="12" t="inlineStr">
@@ -1367,10 +1419,10 @@
         <f>IF(F295="","",F295)</f>
         <v/>
       </c>
-      <c r="C42" s="16" t="n"/>
-      <c r="D42" s="16" t="n"/>
-      <c r="E42" s="16" t="n"/>
-      <c r="F42" s="16" t="n"/>
+      <c r="C42" s="41" t="n"/>
+      <c r="D42" s="41" t="n"/>
+      <c r="E42" s="41" t="n"/>
+      <c r="F42" s="42" t="n"/>
     </row>
     <row r="43" ht="44" customHeight="1">
       <c r="A43" s="17" t="inlineStr">
@@ -1382,11 +1434,13 @@
         <f>IF(F295="","","Αστερίσκοι: "&amp;SUMPRODUCT(LEN(B27:F34)-LEN(SUBSTITUTE(B27:F34,"*","")))&amp;" (το IEEE Xplore δέχεται έως 10 ανά αναζήτηση). "&amp;IF(SUMPRODUCT(--ISNUMBER(FIND("*",B27:F34)),--((ISNUMBER(FIND(" ",TRIM(B27:F34)))+ISNUMBER(FIND("-",B27:F34)))&gt;0))&gt;0,"ΠΡΟΣΟΧΗ: "&amp;SUMPRODUCT(--ISNUMBER(FIND("*",B27:F34)),--((ISNUMBER(FIND(" ",TRIM(B27:F34)))+ISNUMBER(FIND("-",B27:F34)))&gt;0))&amp;" όρος ή όροι έχουν αστερίσκο μέσα σε φράση ή μετά από ενωτικό. Στο ERIC δεν επιστρέφουν αποτελέσματα: γράψτε τις παραλλαγές ολόκληρες.","Κανένας αστερίσκος μέσα σε φράση ή μετά από ενωτικό."))</f>
         <v/>
       </c>
-      <c r="C43" s="16" t="n"/>
-      <c r="D43" s="16" t="n"/>
-      <c r="E43" s="16" t="n"/>
-      <c r="F43" s="16" t="n"/>
-    </row>
+      <c r="C43" s="41" t="n"/>
+      <c r="D43" s="41" t="n"/>
+      <c r="E43" s="41" t="n"/>
+      <c r="F43" s="42" t="n"/>
+    </row>
+    <row r="44"/>
+    <row r="45"/>
     <row r="46" ht="34" customHeight="1">
       <c r="A46" s="25" t="inlineStr">
         <is>
@@ -1401,6 +1455,170 @@
         </is>
       </c>
     </row>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51"/>
+    <row r="52"/>
+    <row r="53"/>
+    <row r="54"/>
+    <row r="55"/>
+    <row r="56"/>
+    <row r="57"/>
+    <row r="58"/>
+    <row r="59"/>
+    <row r="60"/>
+    <row r="61"/>
+    <row r="62"/>
+    <row r="63"/>
+    <row r="64"/>
+    <row r="65"/>
+    <row r="66"/>
+    <row r="67"/>
+    <row r="68"/>
+    <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
+    <row r="73"/>
+    <row r="74"/>
+    <row r="75"/>
+    <row r="76"/>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80"/>
+    <row r="81"/>
+    <row r="82"/>
+    <row r="83"/>
+    <row r="84"/>
+    <row r="85"/>
+    <row r="86"/>
+    <row r="87"/>
+    <row r="88"/>
+    <row r="89"/>
+    <row r="90"/>
+    <row r="91"/>
+    <row r="92"/>
+    <row r="93"/>
+    <row r="94"/>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97"/>
+    <row r="98"/>
+    <row r="99"/>
+    <row r="100"/>
+    <row r="101"/>
+    <row r="102"/>
+    <row r="103"/>
+    <row r="104"/>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107"/>
+    <row r="108"/>
+    <row r="109"/>
+    <row r="110"/>
+    <row r="111"/>
+    <row r="112"/>
+    <row r="113"/>
+    <row r="114"/>
+    <row r="115"/>
+    <row r="116"/>
+    <row r="117"/>
+    <row r="118"/>
+    <row r="119"/>
+    <row r="120"/>
+    <row r="121"/>
+    <row r="122"/>
+    <row r="123"/>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130"/>
+    <row r="131"/>
+    <row r="132"/>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136"/>
+    <row r="137"/>
+    <row r="138"/>
+    <row r="139"/>
+    <row r="140"/>
+    <row r="141"/>
+    <row r="142"/>
+    <row r="143"/>
+    <row r="144"/>
+    <row r="145"/>
+    <row r="146"/>
+    <row r="147"/>
+    <row r="148"/>
+    <row r="149"/>
+    <row r="150"/>
+    <row r="151"/>
+    <row r="152"/>
+    <row r="153"/>
+    <row r="154"/>
+    <row r="155"/>
+    <row r="156"/>
+    <row r="157"/>
+    <row r="158"/>
+    <row r="159"/>
+    <row r="160"/>
+    <row r="161"/>
+    <row r="162"/>
+    <row r="163"/>
+    <row r="164"/>
+    <row r="165"/>
+    <row r="166"/>
+    <row r="167"/>
+    <row r="168"/>
+    <row r="169"/>
+    <row r="170"/>
+    <row r="171"/>
+    <row r="172"/>
+    <row r="173"/>
+    <row r="174"/>
+    <row r="175"/>
+    <row r="176"/>
+    <row r="177"/>
+    <row r="178"/>
+    <row r="179"/>
+    <row r="180"/>
+    <row r="181"/>
+    <row r="182"/>
+    <row r="183"/>
+    <row r="184"/>
+    <row r="185"/>
+    <row r="186"/>
+    <row r="187"/>
+    <row r="188"/>
+    <row r="189"/>
+    <row r="190"/>
+    <row r="191"/>
+    <row r="192"/>
+    <row r="193"/>
+    <row r="194"/>
+    <row r="195"/>
+    <row r="196"/>
+    <row r="197"/>
+    <row r="198"/>
+    <row r="199"/>
+    <row r="200"/>
+    <row r="201"/>
+    <row r="202"/>
+    <row r="203"/>
+    <row r="204"/>
+    <row r="205"/>
+    <row r="206"/>
+    <row r="207"/>
+    <row r="208"/>
+    <row r="209"/>
+    <row r="210"/>
+    <row r="211"/>
     <row r="212" hidden="1">
       <c r="B212">
         <f>IF(TRIM(B6)="","",IF(OR(LEFT(SUBSTITUTE(SUBSTITUTE(TRIM(B6),"“",""""),"”",""""),1)="""",ISERROR(FIND(" ",SUBSTITUTE(SUBSTITUTE(TRIM(B6),"“",""""),"”","""")))),SUBSTITUTE(SUBSTITUTE(TRIM(B6),"“",""""),"”",""""),""""&amp;SUBSTITUTE(SUBSTITUTE(TRIM(B6),"“",""""),"”","""")&amp;""""))</f>
@@ -1577,6 +1795,8 @@
         <v/>
       </c>
     </row>
+    <row r="220"/>
+    <row r="221"/>
     <row r="222" hidden="1">
       <c r="B222">
         <f>B212</f>
@@ -1753,6 +1973,8 @@
         <v/>
       </c>
     </row>
+    <row r="230"/>
+    <row r="231"/>
     <row r="232" hidden="1">
       <c r="B232">
         <f>B14</f>
@@ -1775,6 +1997,48 @@
         <v/>
       </c>
     </row>
+    <row r="233"/>
+    <row r="234"/>
+    <row r="235"/>
+    <row r="236"/>
+    <row r="237"/>
+    <row r="238"/>
+    <row r="239"/>
+    <row r="240"/>
+    <row r="241"/>
+    <row r="242"/>
+    <row r="243"/>
+    <row r="244"/>
+    <row r="245"/>
+    <row r="246"/>
+    <row r="247"/>
+    <row r="248"/>
+    <row r="249"/>
+    <row r="250"/>
+    <row r="251"/>
+    <row r="252"/>
+    <row r="253"/>
+    <row r="254"/>
+    <row r="255"/>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
+    <row r="260"/>
+    <row r="261"/>
+    <row r="262"/>
+    <row r="263"/>
+    <row r="264"/>
+    <row r="265"/>
+    <row r="266"/>
+    <row r="267"/>
+    <row r="268"/>
+    <row r="269"/>
+    <row r="270"/>
+    <row r="271"/>
+    <row r="272"/>
+    <row r="273"/>
+    <row r="274"/>
     <row r="275" hidden="1">
       <c r="B275">
         <f>IF(TRIM(B27)="","",IF(OR(LEFT(SUBSTITUTE(SUBSTITUTE(TRIM(B27),"“",""""),"”",""""),1)="""",ISERROR(FIND(" ",SUBSTITUTE(SUBSTITUTE(TRIM(B27),"“",""""),"”","""")))),SUBSTITUTE(SUBSTITUTE(TRIM(B27),"“",""""),"”",""""),""""&amp;SUBSTITUTE(SUBSTITUTE(TRIM(B27),"“",""""),"”","""")&amp;""""))</f>
@@ -1951,6 +2215,8 @@
         <v/>
       </c>
     </row>
+    <row r="283"/>
+    <row r="284"/>
     <row r="285" hidden="1">
       <c r="B285">
         <f>B275</f>
@@ -2127,6 +2393,8 @@
         <v/>
       </c>
     </row>
+    <row r="293"/>
+    <row r="294"/>
     <row r="295" hidden="1">
       <c r="B295">
         <f>B35</f>
@@ -2198,6 +2466,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -2448,6 +2717,7 @@
       <c r="F25" s="11" t="n"/>
       <c r="G25" s="11" t="n"/>
     </row>
+    <row r="26"/>
     <row r="27">
       <c r="E27" s="28" t="inlineStr">
         <is>
@@ -2507,6 +2777,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -9929,6 +10200,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -10089,6 +10361,8 @@
       </c>
       <c r="D13" s="16" t="n"/>
     </row>
+    <row r="14"/>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="35" t="inlineStr">
         <is>
@@ -10140,6 +10414,8 @@
         <v/>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="35" t="inlineStr">
         <is>
@@ -10269,6 +10545,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -12146,6 +12423,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>
@@ -13667,6 +13945,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="42" customHeight="1">
       <c r="A4" s="27" t="inlineStr">
         <is>

</xml_diff>